<commit_message>
fix(automation): load .env in DailyUpdatePipeline, upgrade night-session cache invalidation & sync latest 2026-10-14 K-bars
</commit_message>
<xml_diff>
--- a/three_strategies_trades_comparison.xlsx
+++ b/three_strategies_trades_comparison.xlsx
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>43102</v>
+        <v>41294</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>17123</v>
+        <v>16505</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>21706</v>
@@ -951,10 +951,10 @@
         </is>
       </c>
       <c r="B17" s="14" t="n">
-        <v>0.4099</v>
+        <v>0.3927</v>
       </c>
       <c r="C17" s="14" t="n">
-        <v>0.1628</v>
+        <v>0.157</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>0.2064</v>
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>0.4333</v>
+        <v>0.4239</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>0.4394</v>
+        <v>0.4328</v>
       </c>
       <c r="D18" s="16" t="n">
         <v>0.4143</v>
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="B19" s="17" t="n">
-        <v>1.76</v>
+        <v>1.71</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="D19" s="17" t="n">
         <v>1.43</v>
@@ -1081,10 +1081,10 @@
         </is>
       </c>
       <c r="B22" s="19" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D22" s="19" t="n">
         <v>70</v>
@@ -1108,12 +1108,12 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>39 / 51</t>
+          <t>39 / 53</t>
         </is>
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
-          <t>29 / 37</t>
+          <t>29 / 38</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
@@ -1165,10 +1165,10 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>1105.411764705882</v>
+        <v>1097.811320754717</v>
       </c>
       <c r="C25" s="21" t="n">
-        <v>1318.540540540541</v>
+        <v>1300.105263157895</v>
       </c>
       <c r="D25" s="21" t="n">
         <v>1240.414634146342</v>
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>148252</v>
+        <v>146444</v>
       </c>
       <c r="C27" s="21" t="n">
-        <v>122273</v>
+        <v>121655</v>
       </c>
       <c r="D27" s="21" t="n">
         <v>126856</v>
@@ -1250,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="101" customWidth="1" min="1" max="1"/>
@@ -1271,7 +1271,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="23" t="inlineStr">
         <is>
-          <t>微台指策略逐筆交易成交稽核表 — 布林_ATR基準 (BB 30/1.8, Pullback 0.4, ATR 14/4) (共計 90 筆交易)</t>
+          <t>微台指策略逐筆交易成交稽核表 — 布林_ATR基準 (BB 30/1.8, Pullback 0.4, ATR 14/4) (共計 92 筆交易)</t>
         </is>
       </c>
     </row>
@@ -5750,6 +5750,104 @@
       </c>
       <c r="M92" s="35" t="n">
         <v>148252</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:40:00</t>
+        </is>
+      </c>
+      <c r="D93" s="25" t="n">
+        <v>48840</v>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:40:00</t>
+        </is>
+      </c>
+      <c r="F93" s="25" t="n">
+        <v>48821</v>
+      </c>
+      <c r="G93" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I93" s="26" t="n">
+        <v>224</v>
+      </c>
+      <c r="J93" s="27" t="n">
+        <v>-984</v>
+      </c>
+      <c r="K93" s="28" t="n">
+        <v>-0.000504</v>
+      </c>
+      <c r="L93" s="38" t="n">
+        <v>42118</v>
+      </c>
+      <c r="M93" s="30" t="n">
+        <v>147268</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:30:00</t>
+        </is>
+      </c>
+      <c r="D94" s="31" t="n">
+        <v>48757</v>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:35:00</t>
+        </is>
+      </c>
+      <c r="F94" s="31" t="n">
+        <v>48772</v>
+      </c>
+      <c r="G94" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H94" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I94" s="19" t="n">
+        <v>224</v>
+      </c>
+      <c r="J94" s="39" t="n">
+        <v>-824</v>
+      </c>
+      <c r="K94" s="40" t="n">
+        <v>-0.000423</v>
+      </c>
+      <c r="L94" s="34" t="n">
+        <v>41294</v>
+      </c>
+      <c r="M94" s="35" t="n">
+        <v>146444</v>
       </c>
     </row>
   </sheetData>
@@ -5766,7 +5864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="103" customWidth="1" min="1" max="1"/>
@@ -5787,7 +5885,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="41" t="inlineStr">
         <is>
-          <t>微台指策略逐筆交易成交稽核表 — 布林_超級趨勢 (BB 30/1.8, Pullback 0.3, ST 10/1.0) (共計 66 筆交易)</t>
+          <t>微台指策略逐筆交易成交稽核表 — 布林_超級趨勢 (BB 30/1.8, Pullback 0.3, ST 10/1.0) (共計 67 筆交易)</t>
         </is>
       </c>
     </row>
@@ -9090,6 +9188,55 @@
       </c>
       <c r="M68" s="35" t="n">
         <v>122273</v>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:30:00</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="n">
+        <v>48757</v>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:35:00</t>
+        </is>
+      </c>
+      <c r="F69" s="25" t="n">
+        <v>48772</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I69" s="26" t="n">
+        <v>168</v>
+      </c>
+      <c r="J69" s="27" t="n">
+        <v>-618</v>
+      </c>
+      <c r="K69" s="28" t="n">
+        <v>-0.000423</v>
+      </c>
+      <c r="L69" s="38" t="n">
+        <v>16505</v>
+      </c>
+      <c r="M69" s="30" t="n">
+        <v>121655</v>
       </c>
     </row>
   </sheetData>
@@ -12598,7 +12745,7 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13 20:25:00</t>
+          <t>2026-10-13 21:20:00</t>
         </is>
       </c>
       <c r="F72" s="31" t="n">
@@ -12609,7 +12756,7 @@
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>期指結算</t>
+          <t>唐奇安破線出場</t>
         </is>
       </c>
       <c r="I72" s="19" t="n">
@@ -12642,7 +12789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1318"/>
+  <dimension ref="A1:E1352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -37690,6 +37837,652 @@
         <v>127444</v>
       </c>
     </row>
+    <row r="1319">
+      <c r="A1319" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 20:35:00</t>
+        </is>
+      </c>
+      <c r="B1319" s="25" t="n">
+        <v>48473</v>
+      </c>
+      <c r="C1319" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1319" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1319" s="25" t="n">
+        <v>127924</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 20:50:00</t>
+        </is>
+      </c>
+      <c r="B1320" s="31" t="n">
+        <v>48468</v>
+      </c>
+      <c r="C1320" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1320" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1320" s="31" t="n">
+        <v>128074</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 21:05:00</t>
+        </is>
+      </c>
+      <c r="B1321" s="25" t="n">
+        <v>48459</v>
+      </c>
+      <c r="C1321" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1321" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1321" s="25" t="n">
+        <v>128344</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 21:20:00</t>
+        </is>
+      </c>
+      <c r="B1322" s="31" t="n">
+        <v>48503</v>
+      </c>
+      <c r="C1322" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1322" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1322" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 21:35:00</t>
+        </is>
+      </c>
+      <c r="B1323" s="25" t="n">
+        <v>48722</v>
+      </c>
+      <c r="C1323" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1323" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1323" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 21:50:00</t>
+        </is>
+      </c>
+      <c r="B1324" s="31" t="n">
+        <v>48740</v>
+      </c>
+      <c r="C1324" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1324" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1324" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 22:05:00</t>
+        </is>
+      </c>
+      <c r="B1325" s="25" t="n">
+        <v>48798</v>
+      </c>
+      <c r="C1325" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1325" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1325" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 22:20:00</t>
+        </is>
+      </c>
+      <c r="B1326" s="31" t="n">
+        <v>48774</v>
+      </c>
+      <c r="C1326" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1326" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1326" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 22:35:00</t>
+        </is>
+      </c>
+      <c r="B1327" s="25" t="n">
+        <v>48757</v>
+      </c>
+      <c r="C1327" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1327" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1327" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 22:50:00</t>
+        </is>
+      </c>
+      <c r="B1328" s="31" t="n">
+        <v>48663</v>
+      </c>
+      <c r="C1328" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1328" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1328" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 23:05:00</t>
+        </is>
+      </c>
+      <c r="B1329" s="25" t="n">
+        <v>48672</v>
+      </c>
+      <c r="C1329" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1329" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1329" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 23:20:00</t>
+        </is>
+      </c>
+      <c r="B1330" s="31" t="n">
+        <v>48649</v>
+      </c>
+      <c r="C1330" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1330" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1330" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 23:35:00</t>
+        </is>
+      </c>
+      <c r="B1331" s="25" t="n">
+        <v>48605</v>
+      </c>
+      <c r="C1331" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1331" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1331" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 23:50:00</t>
+        </is>
+      </c>
+      <c r="B1332" s="31" t="n">
+        <v>48681</v>
+      </c>
+      <c r="C1332" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1332" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1332" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:05:00</t>
+        </is>
+      </c>
+      <c r="B1333" s="25" t="n">
+        <v>48758</v>
+      </c>
+      <c r="C1333" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1333" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1333" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:20:00</t>
+        </is>
+      </c>
+      <c r="B1334" s="31" t="n">
+        <v>48825</v>
+      </c>
+      <c r="C1334" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1334" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1334" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:35:00</t>
+        </is>
+      </c>
+      <c r="B1335" s="25" t="n">
+        <v>48853</v>
+      </c>
+      <c r="C1335" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1335" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1335" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:50:00</t>
+        </is>
+      </c>
+      <c r="B1336" s="31" t="n">
+        <v>48825</v>
+      </c>
+      <c r="C1336" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1336" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1336" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 01:05:00</t>
+        </is>
+      </c>
+      <c r="B1337" s="25" t="n">
+        <v>48770</v>
+      </c>
+      <c r="C1337" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1337" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1337" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 01:20:00</t>
+        </is>
+      </c>
+      <c r="B1338" s="31" t="n">
+        <v>48743</v>
+      </c>
+      <c r="C1338" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1338" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1338" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 01:35:00</t>
+        </is>
+      </c>
+      <c r="B1339" s="25" t="n">
+        <v>48777</v>
+      </c>
+      <c r="C1339" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1339" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1339" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 01:50:00</t>
+        </is>
+      </c>
+      <c r="B1340" s="31" t="n">
+        <v>48714</v>
+      </c>
+      <c r="C1340" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1340" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1340" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 02:05:00</t>
+        </is>
+      </c>
+      <c r="B1341" s="25" t="n">
+        <v>48816</v>
+      </c>
+      <c r="C1341" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1341" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1341" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 02:20:00</t>
+        </is>
+      </c>
+      <c r="B1342" s="31" t="n">
+        <v>48813</v>
+      </c>
+      <c r="C1342" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1342" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1342" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 02:35:00</t>
+        </is>
+      </c>
+      <c r="B1343" s="25" t="n">
+        <v>48790</v>
+      </c>
+      <c r="C1343" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1343" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1343" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 02:50:00</t>
+        </is>
+      </c>
+      <c r="B1344" s="31" t="n">
+        <v>48796</v>
+      </c>
+      <c r="C1344" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1344" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1344" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:05:00</t>
+        </is>
+      </c>
+      <c r="B1345" s="25" t="n">
+        <v>48825</v>
+      </c>
+      <c r="C1345" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1345" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1345" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:20:00</t>
+        </is>
+      </c>
+      <c r="B1346" s="31" t="n">
+        <v>48815</v>
+      </c>
+      <c r="C1346" s="31" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1346" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1346" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:35:00</t>
+        </is>
+      </c>
+      <c r="B1347" s="25" t="n">
+        <v>48843</v>
+      </c>
+      <c r="C1347" s="25" t="n">
+        <v>148252</v>
+      </c>
+      <c r="D1347" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1347" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 03:50:00</t>
+        </is>
+      </c>
+      <c r="B1348" s="31" t="n">
+        <v>48817</v>
+      </c>
+      <c r="C1348" s="31" t="n">
+        <v>147268</v>
+      </c>
+      <c r="D1348" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1348" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:05:00</t>
+        </is>
+      </c>
+      <c r="B1349" s="25" t="n">
+        <v>48817</v>
+      </c>
+      <c r="C1349" s="25" t="n">
+        <v>147268</v>
+      </c>
+      <c r="D1349" s="25" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1349" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:20:00</t>
+        </is>
+      </c>
+      <c r="B1350" s="31" t="n">
+        <v>48754</v>
+      </c>
+      <c r="C1350" s="31" t="n">
+        <v>147268</v>
+      </c>
+      <c r="D1350" s="31" t="n">
+        <v>122273</v>
+      </c>
+      <c r="E1350" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:35:00</t>
+        </is>
+      </c>
+      <c r="B1351" s="25" t="n">
+        <v>48776</v>
+      </c>
+      <c r="C1351" s="25" t="n">
+        <v>146444</v>
+      </c>
+      <c r="D1351" s="25" t="n">
+        <v>121655</v>
+      </c>
+      <c r="E1351" s="25" t="n">
+        <v>126856</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:50:00</t>
+        </is>
+      </c>
+      <c r="B1352" s="31" t="n">
+        <v>48773</v>
+      </c>
+      <c r="C1352" s="31" t="n">
+        <v>146444</v>
+      </c>
+      <c r="D1352" s="31" t="n">
+        <v>121655</v>
+      </c>
+      <c r="E1352" s="31" t="n">
+        <v>126856</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
feat(data): complete 100% TMF history backfill (2024-07-29 to 2026-10-23, 20.05M second bars) & update dashboard
</commit_message>
<xml_diff>
--- a/three_strategies_trades_comparison.xlsx
+++ b/three_strategies_trades_comparison.xlsx
@@ -263,11 +263,11 @@
     <xf numFmtId="169" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>3005</v>
+        <v>3434</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>-23057</v>
+        <v>-22997</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>-8660</v>
+        <v>-15314</v>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="B17" s="14" t="n">
-        <v>0.0286</v>
+        <v>0.0327</v>
       </c>
       <c r="C17" s="14" t="n">
-        <v>-0.2193</v>
+        <v>-0.2187</v>
       </c>
       <c r="D17" s="14" t="n">
-        <v>-0.0824</v>
+        <v>-0.1456</v>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>0.4011</v>
+        <v>0.3958</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>0.3214</v>
+        <v>0.3133</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>0.3478</v>
+        <v>0.3333</v>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
@@ -1009,10 +1009,10 @@
         <v>1.03</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="D19" s="17" t="n">
-        <v>0.91</v>
+        <v>0.86</v>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
@@ -1035,10 +1035,10 @@
         <v>-31940</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>-50763</v>
+        <v>-55109</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>-34757</v>
+        <v>-42197</v>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
@@ -1061,10 +1061,10 @@
         <v>0.2383</v>
       </c>
       <c r="C21" s="18" t="n">
-        <v>0.3837</v>
+        <v>0.4166</v>
       </c>
       <c r="D21" s="18" t="n">
-        <v>0.2671</v>
+        <v>0.3243</v>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="B22" s="19" t="n">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D22" s="19" t="n">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
@@ -1111,17 +1111,17 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>71 / 106</t>
+          <t>76 / 116</t>
         </is>
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
-          <t>45 / 95</t>
+          <t>47 / 103</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
         <is>
-          <t>48 / 90</t>
+          <t>50 / 100</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -1142,13 +1142,13 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>1546.267605633803</v>
+        <v>1599.144736842105</v>
       </c>
       <c r="C24" s="12" t="n">
-        <v>1757.822222222222</v>
+        <v>1884.893617021277</v>
       </c>
       <c r="D24" s="12" t="n">
-        <v>1797.354166666667</v>
+        <v>1918.3</v>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
@@ -1168,13 +1168,13 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>1007.358490566038</v>
+        <v>1018.112068965517</v>
       </c>
       <c r="C25" s="21" t="n">
-        <v>1075.357894736842</v>
+        <v>1083.368932038835</v>
       </c>
       <c r="D25" s="21" t="n">
-        <v>1054.811111111111</v>
+        <v>1112.29</v>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
@@ -1220,13 +1220,13 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>108155</v>
+        <v>108584</v>
       </c>
       <c r="C27" s="21" t="n">
-        <v>82093</v>
+        <v>82153</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>96490</v>
+        <v>89836</v>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M179"/>
+  <dimension ref="A1:M194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="102" customWidth="1" min="1" max="1"/>
@@ -1274,7 +1274,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="23" t="inlineStr">
         <is>
-          <t>微台指策略逐筆交易成交稽核表 — 布林_ATR基準 (BB 30/1.8, Pullback 0.4, ATR 14/4) (共計 177 筆交易)</t>
+          <t>微台指策略逐筆交易成交稽核表 — 布林_ATR基準 (BB 30/1.8, Pullback 0.4, ATR 14/4) (共計 192 筆交易)</t>
         </is>
       </c>
     </row>
@@ -10016,6 +10016,741 @@
       </c>
       <c r="M179" s="30" t="n">
         <v>108155</v>
+      </c>
+    </row>
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="8" t="n">
+        <v>178</v>
+      </c>
+      <c r="B180" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C180" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:30:00</t>
+        </is>
+      </c>
+      <c r="D180" s="31" t="n">
+        <v>47211</v>
+      </c>
+      <c r="E180" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:55:00</t>
+        </is>
+      </c>
+      <c r="F180" s="31" t="n">
+        <v>47111</v>
+      </c>
+      <c r="G180" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H180" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I180" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J180" s="39" t="n">
+        <v>-2110</v>
+      </c>
+      <c r="K180" s="40" t="n">
+        <v>-0.002235</v>
+      </c>
+      <c r="L180" s="34" t="n">
+        <v>895</v>
+      </c>
+      <c r="M180" s="35" t="n">
+        <v>106045</v>
+      </c>
+    </row>
+    <row r="181" ht="20" customHeight="1">
+      <c r="A181" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:10:00</t>
+        </is>
+      </c>
+      <c r="D181" s="25" t="n">
+        <v>47245</v>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:20:00</t>
+        </is>
+      </c>
+      <c r="F181" s="25" t="n">
+        <v>47251</v>
+      </c>
+      <c r="G181" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H181" s="5" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I181" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J181" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="K181" s="37" t="n">
+        <v>1.1e-05</v>
+      </c>
+      <c r="L181" s="38" t="n">
+        <v>905</v>
+      </c>
+      <c r="M181" s="30" t="n">
+        <v>106055</v>
+      </c>
+    </row>
+    <row r="182" ht="20" customHeight="1">
+      <c r="A182" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="B182" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:10:00</t>
+        </is>
+      </c>
+      <c r="D182" s="31" t="n">
+        <v>47340</v>
+      </c>
+      <c r="E182" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:15:00</t>
+        </is>
+      </c>
+      <c r="F182" s="31" t="n">
+        <v>47379</v>
+      </c>
+      <c r="G182" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H182" s="8" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I182" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J182" s="32" t="n">
+        <v>670</v>
+      </c>
+      <c r="K182" s="33" t="n">
+        <v>0.000708</v>
+      </c>
+      <c r="L182" s="34" t="n">
+        <v>1575</v>
+      </c>
+      <c r="M182" s="35" t="n">
+        <v>106725</v>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="A183" s="5" t="n">
+        <v>181</v>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:25:00</t>
+        </is>
+      </c>
+      <c r="D183" s="25" t="n">
+        <v>47394</v>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:35:00</t>
+        </is>
+      </c>
+      <c r="F183" s="25" t="n">
+        <v>47342</v>
+      </c>
+      <c r="G183" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H183" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I183" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J183" s="27" t="n">
+        <v>-1150</v>
+      </c>
+      <c r="K183" s="28" t="n">
+        <v>-0.001213</v>
+      </c>
+      <c r="L183" s="38" t="n">
+        <v>425</v>
+      </c>
+      <c r="M183" s="30" t="n">
+        <v>105575</v>
+      </c>
+    </row>
+    <row r="184" ht="20" customHeight="1">
+      <c r="A184" s="8" t="n">
+        <v>182</v>
+      </c>
+      <c r="B184" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:45:00</t>
+        </is>
+      </c>
+      <c r="D184" s="31" t="n">
+        <v>47439</v>
+      </c>
+      <c r="E184" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:55:00</t>
+        </is>
+      </c>
+      <c r="F184" s="31" t="n">
+        <v>47463</v>
+      </c>
+      <c r="G184" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H184" s="8" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I184" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J184" s="32" t="n">
+        <v>370</v>
+      </c>
+      <c r="K184" s="33" t="n">
+        <v>0.00039</v>
+      </c>
+      <c r="L184" s="34" t="n">
+        <v>795</v>
+      </c>
+      <c r="M184" s="35" t="n">
+        <v>105945</v>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="5" t="n">
+        <v>183</v>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:15:00</t>
+        </is>
+      </c>
+      <c r="D185" s="25" t="n">
+        <v>47515</v>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:25:00</t>
+        </is>
+      </c>
+      <c r="F185" s="25" t="n">
+        <v>47476</v>
+      </c>
+      <c r="G185" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I185" s="26" t="n">
+        <v>111</v>
+      </c>
+      <c r="J185" s="27" t="n">
+        <v>-891</v>
+      </c>
+      <c r="K185" s="28" t="n">
+        <v>-0.0009379999999999999</v>
+      </c>
+      <c r="L185" s="29" t="n">
+        <v>-96</v>
+      </c>
+      <c r="M185" s="30" t="n">
+        <v>105054</v>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="8" t="n">
+        <v>184</v>
+      </c>
+      <c r="B186" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:10:00</t>
+        </is>
+      </c>
+      <c r="D186" s="31" t="n">
+        <v>47300</v>
+      </c>
+      <c r="E186" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:15:00</t>
+        </is>
+      </c>
+      <c r="F186" s="31" t="n">
+        <v>47364</v>
+      </c>
+      <c r="G186" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I186" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J186" s="39" t="n">
+        <v>-1390</v>
+      </c>
+      <c r="K186" s="40" t="n">
+        <v>-0.001469</v>
+      </c>
+      <c r="L186" s="41" t="n">
+        <v>-1486</v>
+      </c>
+      <c r="M186" s="35" t="n">
+        <v>103664</v>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:25:00</t>
+        </is>
+      </c>
+      <c r="D187" s="25" t="n">
+        <v>47137</v>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:15:00</t>
+        </is>
+      </c>
+      <c r="F187" s="25" t="n">
+        <v>46912</v>
+      </c>
+      <c r="G187" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I187" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J187" s="36" t="n">
+        <v>4390</v>
+      </c>
+      <c r="K187" s="37" t="n">
+        <v>0.004657</v>
+      </c>
+      <c r="L187" s="38" t="n">
+        <v>2904</v>
+      </c>
+      <c r="M187" s="30" t="n">
+        <v>108054</v>
+      </c>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="A188" s="8" t="n">
+        <v>186</v>
+      </c>
+      <c r="B188" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C188" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:15:00</t>
+        </is>
+      </c>
+      <c r="D188" s="31" t="n">
+        <v>46165</v>
+      </c>
+      <c r="E188" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:15:00</t>
+        </is>
+      </c>
+      <c r="F188" s="31" t="n">
+        <v>46211</v>
+      </c>
+      <c r="G188" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H188" s="8" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I188" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J188" s="39" t="n">
+        <v>-1030</v>
+      </c>
+      <c r="K188" s="40" t="n">
+        <v>-0.001116</v>
+      </c>
+      <c r="L188" s="34" t="n">
+        <v>1874</v>
+      </c>
+      <c r="M188" s="35" t="n">
+        <v>107024</v>
+      </c>
+    </row>
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="5" t="n">
+        <v>187</v>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:00:00</t>
+        </is>
+      </c>
+      <c r="D189" s="25" t="n">
+        <v>46050</v>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:05:00</t>
+        </is>
+      </c>
+      <c r="F189" s="25" t="n">
+        <v>46085</v>
+      </c>
+      <c r="G189" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I189" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J189" s="27" t="n">
+        <v>-810</v>
+      </c>
+      <c r="K189" s="28" t="n">
+        <v>-0.000879</v>
+      </c>
+      <c r="L189" s="38" t="n">
+        <v>1064</v>
+      </c>
+      <c r="M189" s="30" t="n">
+        <v>106214</v>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="8" t="n">
+        <v>188</v>
+      </c>
+      <c r="B190" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C190" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="D190" s="31" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E190" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="F190" s="31" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G190" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H190" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I190" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J190" s="39" t="n">
+        <v>-1690</v>
+      </c>
+      <c r="K190" s="40" t="n">
+        <v>-0.001825</v>
+      </c>
+      <c r="L190" s="41" t="n">
+        <v>-626</v>
+      </c>
+      <c r="M190" s="35" t="n">
+        <v>104524</v>
+      </c>
+    </row>
+    <row r="191" ht="20" customHeight="1">
+      <c r="A191" s="5" t="n">
+        <v>189</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:30:00</t>
+        </is>
+      </c>
+      <c r="D191" s="25" t="n">
+        <v>46077</v>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:10:00</t>
+        </is>
+      </c>
+      <c r="F191" s="25" t="n">
+        <v>45756</v>
+      </c>
+      <c r="G191" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I191" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J191" s="36" t="n">
+        <v>6310</v>
+      </c>
+      <c r="K191" s="37" t="n">
+        <v>0.006847</v>
+      </c>
+      <c r="L191" s="38" t="n">
+        <v>5684</v>
+      </c>
+      <c r="M191" s="30" t="n">
+        <v>110834</v>
+      </c>
+    </row>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="8" t="n">
+        <v>190</v>
+      </c>
+      <c r="B192" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C192" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:55:00</t>
+        </is>
+      </c>
+      <c r="D192" s="31" t="n">
+        <v>45688</v>
+      </c>
+      <c r="E192" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:55:00</t>
+        </is>
+      </c>
+      <c r="F192" s="31" t="n">
+        <v>45714</v>
+      </c>
+      <c r="G192" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H192" s="8" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I192" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J192" s="39" t="n">
+        <v>-630</v>
+      </c>
+      <c r="K192" s="40" t="n">
+        <v>-0.0006890000000000001</v>
+      </c>
+      <c r="L192" s="34" t="n">
+        <v>5054</v>
+      </c>
+      <c r="M192" s="35" t="n">
+        <v>110204</v>
+      </c>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="A193" s="5" t="n">
+        <v>191</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:10:00</t>
+        </is>
+      </c>
+      <c r="D193" s="25" t="n">
+        <v>45660</v>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:15:00</t>
+        </is>
+      </c>
+      <c r="F193" s="25" t="n">
+        <v>45727</v>
+      </c>
+      <c r="G193" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I193" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J193" s="27" t="n">
+        <v>-1450</v>
+      </c>
+      <c r="K193" s="28" t="n">
+        <v>-0.001588</v>
+      </c>
+      <c r="L193" s="38" t="n">
+        <v>3604</v>
+      </c>
+      <c r="M193" s="30" t="n">
+        <v>108754</v>
+      </c>
+    </row>
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C194" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:05:00</t>
+        </is>
+      </c>
+      <c r="D194" s="31" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E194" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:05:00</t>
+        </is>
+      </c>
+      <c r="F194" s="31" t="n">
+        <v>45585</v>
+      </c>
+      <c r="G194" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H194" s="8" t="inlineStr">
+        <is>
+          <t>ATR均線停利</t>
+        </is>
+      </c>
+      <c r="I194" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J194" s="39" t="n">
+        <v>-170</v>
+      </c>
+      <c r="K194" s="40" t="n">
+        <v>-0.000186</v>
+      </c>
+      <c r="L194" s="34" t="n">
+        <v>3434</v>
+      </c>
+      <c r="M194" s="35" t="n">
+        <v>108584</v>
       </c>
     </row>
   </sheetData>
@@ -10032,7 +10767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M142"/>
+  <dimension ref="A1:M152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -10051,9 +10786,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>微台指策略逐筆交易成交稽核表 — 布林_超級趨勢 (BB 30/1.8, Pullback 0.3, ST 10/1.0) (共計 140 筆交易)</t>
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>微台指策略逐筆交易成交稽核表 — 布林_超級趨勢 (BB 30/1.8, Pullback 0.3, ST 10/1.0) (共計 150 筆交易)</t>
         </is>
       </c>
     </row>
@@ -15801,7 +16536,7 @@
       <c r="K118" s="40" t="n">
         <v>-0.002503</v>
       </c>
-      <c r="L118" s="42" t="n">
+      <c r="L118" s="41" t="n">
         <v>-1442</v>
       </c>
       <c r="M118" s="35" t="n">
@@ -15899,7 +16634,7 @@
       <c r="K120" s="40" t="n">
         <v>-0.004996</v>
       </c>
-      <c r="L120" s="42" t="n">
+      <c r="L120" s="41" t="n">
         <v>-8682</v>
       </c>
       <c r="M120" s="35" t="n">
@@ -15997,7 +16732,7 @@
       <c r="K122" s="40" t="n">
         <v>-0.001688</v>
       </c>
-      <c r="L122" s="42" t="n">
+      <c r="L122" s="41" t="n">
         <v>-12943</v>
       </c>
       <c r="M122" s="35" t="n">
@@ -16095,7 +16830,7 @@
       <c r="K124" s="40" t="n">
         <v>-0.001069</v>
       </c>
-      <c r="L124" s="42" t="n">
+      <c r="L124" s="41" t="n">
         <v>-14729</v>
       </c>
       <c r="M124" s="35" t="n">
@@ -16193,7 +16928,7 @@
       <c r="K126" s="40" t="n">
         <v>-0.00012</v>
       </c>
-      <c r="L126" s="42" t="n">
+      <c r="L126" s="41" t="n">
         <v>-15651</v>
       </c>
       <c r="M126" s="35" t="n">
@@ -16291,7 +17026,7 @@
       <c r="K128" s="40" t="n">
         <v>-0.003613</v>
       </c>
-      <c r="L128" s="42" t="n">
+      <c r="L128" s="41" t="n">
         <v>-19063</v>
       </c>
       <c r="M128" s="35" t="n">
@@ -16389,7 +17124,7 @@
       <c r="K130" s="40" t="n">
         <v>-0.0008219999999999999</v>
       </c>
-      <c r="L130" s="42" t="n">
+      <c r="L130" s="41" t="n">
         <v>-19385</v>
       </c>
       <c r="M130" s="35" t="n">
@@ -16487,7 +17222,7 @@
       <c r="K132" s="40" t="n">
         <v>-0.001253</v>
       </c>
-      <c r="L132" s="42" t="n">
+      <c r="L132" s="41" t="n">
         <v>-20407</v>
       </c>
       <c r="M132" s="35" t="n">
@@ -16585,7 +17320,7 @@
       <c r="K134" s="40" t="n">
         <v>-0.005046</v>
       </c>
-      <c r="L134" s="42" t="n">
+      <c r="L134" s="41" t="n">
         <v>-23019</v>
       </c>
       <c r="M134" s="35" t="n">
@@ -16683,7 +17418,7 @@
       <c r="K136" s="40" t="n">
         <v>-0.001266</v>
       </c>
-      <c r="L136" s="42" t="n">
+      <c r="L136" s="41" t="n">
         <v>-20641</v>
       </c>
       <c r="M136" s="35" t="n">
@@ -16781,7 +17516,7 @@
       <c r="K138" s="40" t="n">
         <v>-0.001658</v>
       </c>
-      <c r="L138" s="42" t="n">
+      <c r="L138" s="41" t="n">
         <v>-21653</v>
       </c>
       <c r="M138" s="35" t="n">
@@ -16879,7 +17614,7 @@
       <c r="K140" s="40" t="n">
         <v>-0.001602</v>
       </c>
-      <c r="L140" s="42" t="n">
+      <c r="L140" s="41" t="n">
         <v>-23625</v>
       </c>
       <c r="M140" s="35" t="n">
@@ -16954,34 +17689,524 @@
       </c>
       <c r="E142" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21 13:25:00</t>
+          <t>2026-10-21 15:00:00</t>
         </is>
       </c>
       <c r="F142" s="31" t="n">
-        <v>46650</v>
+        <v>47003</v>
       </c>
       <c r="G142" s="8" t="n">
         <v>1</v>
       </c>
       <c r="H142" s="8" t="inlineStr">
         <is>
-          <t>期指結算</t>
+          <t>停損 (SL)</t>
         </is>
       </c>
       <c r="I142" s="19" t="n">
         <v>56</v>
       </c>
-      <c r="J142" s="32" t="n">
-        <v>44</v>
-      </c>
-      <c r="K142" s="33" t="n">
-        <v>9.400000000000001e-05</v>
-      </c>
-      <c r="L142" s="42" t="n">
-        <v>-23057</v>
+      <c r="J142" s="39" t="n">
+        <v>-3486</v>
+      </c>
+      <c r="K142" s="40" t="n">
+        <v>-0.007471</v>
+      </c>
+      <c r="L142" s="41" t="n">
+        <v>-26587</v>
       </c>
       <c r="M142" s="35" t="n">
-        <v>82093</v>
+        <v>78563</v>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="5" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:30:00</t>
+        </is>
+      </c>
+      <c r="D143" s="25" t="n">
+        <v>47211</v>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:15:00</t>
+        </is>
+      </c>
+      <c r="F143" s="25" t="n">
+        <v>47254</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>超級趨勢出場</t>
+        </is>
+      </c>
+      <c r="I143" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J143" s="36" t="n">
+        <v>374</v>
+      </c>
+      <c r="K143" s="37" t="n">
+        <v>0.0007920000000000001</v>
+      </c>
+      <c r="L143" s="29" t="n">
+        <v>-26213</v>
+      </c>
+      <c r="M143" s="30" t="n">
+        <v>78937</v>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:20:00</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="n">
+        <v>47379</v>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:35:00</t>
+        </is>
+      </c>
+      <c r="F144" s="31" t="n">
+        <v>47326</v>
+      </c>
+      <c r="G144" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I144" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J144" s="39" t="n">
+        <v>-586</v>
+      </c>
+      <c r="K144" s="40" t="n">
+        <v>-0.001237</v>
+      </c>
+      <c r="L144" s="41" t="n">
+        <v>-26799</v>
+      </c>
+      <c r="M144" s="35" t="n">
+        <v>78351</v>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:15:00</t>
+        </is>
+      </c>
+      <c r="D145" s="25" t="n">
+        <v>47515</v>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:25:00</t>
+        </is>
+      </c>
+      <c r="F145" s="25" t="n">
+        <v>47476</v>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I145" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J145" s="27" t="n">
+        <v>-446</v>
+      </c>
+      <c r="K145" s="28" t="n">
+        <v>-0.0009389999999999999</v>
+      </c>
+      <c r="L145" s="29" t="n">
+        <v>-27245</v>
+      </c>
+      <c r="M145" s="30" t="n">
+        <v>77905</v>
+      </c>
+    </row>
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="8" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:10:00</t>
+        </is>
+      </c>
+      <c r="D146" s="31" t="n">
+        <v>47300</v>
+      </c>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:15:00</t>
+        </is>
+      </c>
+      <c r="F146" s="31" t="n">
+        <v>47364</v>
+      </c>
+      <c r="G146" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I146" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J146" s="39" t="n">
+        <v>-696</v>
+      </c>
+      <c r="K146" s="40" t="n">
+        <v>-0.001471</v>
+      </c>
+      <c r="L146" s="41" t="n">
+        <v>-27941</v>
+      </c>
+      <c r="M146" s="35" t="n">
+        <v>77209</v>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="A147" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:45:00</t>
+        </is>
+      </c>
+      <c r="D147" s="25" t="n">
+        <v>47041</v>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:20:00</t>
+        </is>
+      </c>
+      <c r="F147" s="25" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>超級趨勢出場</t>
+        </is>
+      </c>
+      <c r="I147" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J147" s="36" t="n">
+        <v>7364</v>
+      </c>
+      <c r="K147" s="37" t="n">
+        <v>0.015654</v>
+      </c>
+      <c r="L147" s="29" t="n">
+        <v>-20577</v>
+      </c>
+      <c r="M147" s="30" t="n">
+        <v>84573</v>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1">
+      <c r="A148" s="8" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:00:00</t>
+        </is>
+      </c>
+      <c r="D148" s="31" t="n">
+        <v>46050</v>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:10:00</t>
+        </is>
+      </c>
+      <c r="F148" s="31" t="n">
+        <v>46227</v>
+      </c>
+      <c r="G148" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I148" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J148" s="39" t="n">
+        <v>-1826</v>
+      </c>
+      <c r="K148" s="40" t="n">
+        <v>-0.003965</v>
+      </c>
+      <c r="L148" s="41" t="n">
+        <v>-22403</v>
+      </c>
+      <c r="M148" s="35" t="n">
+        <v>82747</v>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="D149" s="25" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="F149" s="25" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I149" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J149" s="27" t="n">
+        <v>-846</v>
+      </c>
+      <c r="K149" s="28" t="n">
+        <v>-0.001827</v>
+      </c>
+      <c r="L149" s="29" t="n">
+        <v>-23249</v>
+      </c>
+      <c r="M149" s="30" t="n">
+        <v>81901</v>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:30:00</t>
+        </is>
+      </c>
+      <c r="D150" s="31" t="n">
+        <v>46077</v>
+      </c>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:20:00</t>
+        </is>
+      </c>
+      <c r="F150" s="31" t="n">
+        <v>45892</v>
+      </c>
+      <c r="G150" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t>超級趨勢出場</t>
+        </is>
+      </c>
+      <c r="I150" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J150" s="32" t="n">
+        <v>1794</v>
+      </c>
+      <c r="K150" s="33" t="n">
+        <v>0.003893</v>
+      </c>
+      <c r="L150" s="41" t="n">
+        <v>-21455</v>
+      </c>
+      <c r="M150" s="35" t="n">
+        <v>83695</v>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1">
+      <c r="A151" s="5" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:55:00</t>
+        </is>
+      </c>
+      <c r="D151" s="25" t="n">
+        <v>45688</v>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:30:00</t>
+        </is>
+      </c>
+      <c r="F151" s="25" t="n">
+        <v>45771</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H151" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I151" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J151" s="27" t="n">
+        <v>-886</v>
+      </c>
+      <c r="K151" s="28" t="n">
+        <v>-0.001939</v>
+      </c>
+      <c r="L151" s="29" t="n">
+        <v>-22341</v>
+      </c>
+      <c r="M151" s="30" t="n">
+        <v>82809</v>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1">
+      <c r="A152" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:05:00</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:10:00</t>
+        </is>
+      </c>
+      <c r="F152" s="31" t="n">
+        <v>45642</v>
+      </c>
+      <c r="G152" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H152" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I152" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J152" s="39" t="n">
+        <v>-656</v>
+      </c>
+      <c r="K152" s="40" t="n">
+        <v>-0.001439</v>
+      </c>
+      <c r="L152" s="41" t="n">
+        <v>-22997</v>
+      </c>
+      <c r="M152" s="35" t="n">
+        <v>82153</v>
       </c>
     </row>
   </sheetData>
@@ -16998,7 +18223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M140"/>
+  <dimension ref="A1:M152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -17019,7 +18244,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>微台指策略逐筆交易成交稽核表 — 布林_唐奇安 (BB 31/1.75, Pullback 0.3, Donchian 2) (共計 138 筆交易)</t>
+          <t>微台指策略逐筆交易成交稽核表 — 布林_唐奇安 (BB 31/1.75, Pullback 0.3, Donchian 2) (共計 150 筆交易)</t>
         </is>
       </c>
     </row>
@@ -23453,7 +24678,7 @@
       <c r="K132" s="40" t="n">
         <v>-0.001251</v>
       </c>
-      <c r="L132" s="42" t="n">
+      <c r="L132" s="41" t="n">
         <v>-940</v>
       </c>
       <c r="M132" s="35" t="n">
@@ -23551,7 +24776,7 @@
       <c r="K134" s="40" t="n">
         <v>-0.005044</v>
       </c>
-      <c r="L134" s="42" t="n">
+      <c r="L134" s="41" t="n">
         <v>-6160</v>
       </c>
       <c r="M134" s="35" t="n">
@@ -23649,7 +24874,7 @@
       <c r="K136" s="40" t="n">
         <v>-0.0009840000000000001</v>
       </c>
-      <c r="L136" s="42" t="n">
+      <c r="L136" s="41" t="n">
         <v>-5640</v>
       </c>
       <c r="M136" s="35" t="n">
@@ -23747,7 +24972,7 @@
       <c r="K138" s="40" t="n">
         <v>-0.000858</v>
       </c>
-      <c r="L138" s="42" t="n">
+      <c r="L138" s="41" t="n">
         <v>-9800</v>
       </c>
       <c r="M138" s="35" t="n">
@@ -23822,34 +25047,622 @@
       </c>
       <c r="E140" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21 13:25:00</t>
+          <t>2026-10-21 15:00:00</t>
         </is>
       </c>
       <c r="F140" s="31" t="n">
-        <v>46650</v>
+        <v>47003</v>
       </c>
       <c r="G140" s="8" t="n">
         <v>2</v>
       </c>
       <c r="H140" s="8" t="inlineStr">
         <is>
-          <t>期指結算</t>
+          <t>停損 (SL)</t>
         </is>
       </c>
       <c r="I140" s="19" t="n">
         <v>110</v>
       </c>
-      <c r="J140" s="32" t="n">
-        <v>90</v>
-      </c>
-      <c r="K140" s="33" t="n">
-        <v>9.599999999999999e-05</v>
-      </c>
-      <c r="L140" s="42" t="n">
-        <v>-8660</v>
+      <c r="J140" s="39" t="n">
+        <v>-6970</v>
+      </c>
+      <c r="K140" s="40" t="n">
+        <v>-0.007469</v>
+      </c>
+      <c r="L140" s="41" t="n">
+        <v>-15720</v>
       </c>
       <c r="M140" s="35" t="n">
-        <v>96490</v>
+        <v>89430</v>
+      </c>
+    </row>
+    <row r="141" ht="20" customHeight="1">
+      <c r="A141" s="5" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:30:00</t>
+        </is>
+      </c>
+      <c r="D141" s="25" t="n">
+        <v>47211</v>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:05:00</t>
+        </is>
+      </c>
+      <c r="F141" s="25" t="n">
+        <v>47274</v>
+      </c>
+      <c r="G141" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>唐奇安破線出場</t>
+        </is>
+      </c>
+      <c r="I141" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J141" s="36" t="n">
+        <v>574</v>
+      </c>
+      <c r="K141" s="37" t="n">
+        <v>0.001216</v>
+      </c>
+      <c r="L141" s="29" t="n">
+        <v>-15146</v>
+      </c>
+      <c r="M141" s="30" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="8" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:20:00</t>
+        </is>
+      </c>
+      <c r="D142" s="31" t="n">
+        <v>47379</v>
+      </c>
+      <c r="E142" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:35:00</t>
+        </is>
+      </c>
+      <c r="F142" s="31" t="n">
+        <v>47326</v>
+      </c>
+      <c r="G142" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H142" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I142" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J142" s="39" t="n">
+        <v>-586</v>
+      </c>
+      <c r="K142" s="40" t="n">
+        <v>-0.001237</v>
+      </c>
+      <c r="L142" s="41" t="n">
+        <v>-15732</v>
+      </c>
+      <c r="M142" s="35" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="5" t="n">
+        <v>141</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 23:45:00</t>
+        </is>
+      </c>
+      <c r="D143" s="25" t="n">
+        <v>47402</v>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:05:00</t>
+        </is>
+      </c>
+      <c r="F143" s="25" t="n">
+        <v>47365</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I143" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J143" s="27" t="n">
+        <v>-426</v>
+      </c>
+      <c r="K143" s="28" t="n">
+        <v>-0.000899</v>
+      </c>
+      <c r="L143" s="29" t="n">
+        <v>-16158</v>
+      </c>
+      <c r="M143" s="30" t="n">
+        <v>88992</v>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:10:00</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="n">
+        <v>47518</v>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:20:00</t>
+        </is>
+      </c>
+      <c r="F144" s="31" t="n">
+        <v>47488</v>
+      </c>
+      <c r="G144" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
+        <is>
+          <t>唐奇安破線出場</t>
+        </is>
+      </c>
+      <c r="I144" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J144" s="39" t="n">
+        <v>-356</v>
+      </c>
+      <c r="K144" s="40" t="n">
+        <v>-0.000749</v>
+      </c>
+      <c r="L144" s="41" t="n">
+        <v>-16514</v>
+      </c>
+      <c r="M144" s="35" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:10:00</t>
+        </is>
+      </c>
+      <c r="D145" s="25" t="n">
+        <v>47300</v>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:15:00</t>
+        </is>
+      </c>
+      <c r="F145" s="25" t="n">
+        <v>47364</v>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I145" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J145" s="27" t="n">
+        <v>-696</v>
+      </c>
+      <c r="K145" s="28" t="n">
+        <v>-0.001471</v>
+      </c>
+      <c r="L145" s="29" t="n">
+        <v>-17210</v>
+      </c>
+      <c r="M145" s="30" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="8" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:45:00</t>
+        </is>
+      </c>
+      <c r="D146" s="31" t="n">
+        <v>47041</v>
+      </c>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:20:00</t>
+        </is>
+      </c>
+      <c r="F146" s="31" t="n">
+        <v>46299</v>
+      </c>
+      <c r="G146" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" s="8" t="inlineStr">
+        <is>
+          <t>唐奇安破線出場</t>
+        </is>
+      </c>
+      <c r="I146" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J146" s="32" t="n">
+        <v>7364</v>
+      </c>
+      <c r="K146" s="33" t="n">
+        <v>0.015654</v>
+      </c>
+      <c r="L146" s="41" t="n">
+        <v>-9846</v>
+      </c>
+      <c r="M146" s="35" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="A147" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:00:00</t>
+        </is>
+      </c>
+      <c r="D147" s="25" t="n">
+        <v>46050</v>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:10:00</t>
+        </is>
+      </c>
+      <c r="F147" s="25" t="n">
+        <v>46227</v>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I147" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="J147" s="27" t="n">
+        <v>-3650</v>
+      </c>
+      <c r="K147" s="28" t="n">
+        <v>-0.003963</v>
+      </c>
+      <c r="L147" s="29" t="n">
+        <v>-13496</v>
+      </c>
+      <c r="M147" s="30" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1">
+      <c r="A148" s="8" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>做多 (BUY)</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="D148" s="31" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:40:00</t>
+        </is>
+      </c>
+      <c r="F148" s="31" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G148" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I148" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J148" s="39" t="n">
+        <v>-1690</v>
+      </c>
+      <c r="K148" s="40" t="n">
+        <v>-0.001825</v>
+      </c>
+      <c r="L148" s="41" t="n">
+        <v>-15186</v>
+      </c>
+      <c r="M148" s="35" t="n">
+        <v>89964</v>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:30:00</t>
+        </is>
+      </c>
+      <c r="D149" s="25" t="n">
+        <v>46077</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:20:00</t>
+        </is>
+      </c>
+      <c r="F149" s="25" t="n">
+        <v>45892</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>唐奇安破線出場</t>
+        </is>
+      </c>
+      <c r="I149" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J149" s="36" t="n">
+        <v>1794</v>
+      </c>
+      <c r="K149" s="37" t="n">
+        <v>0.003893</v>
+      </c>
+      <c r="L149" s="29" t="n">
+        <v>-13392</v>
+      </c>
+      <c r="M149" s="30" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:55:00</t>
+        </is>
+      </c>
+      <c r="D150" s="31" t="n">
+        <v>45688</v>
+      </c>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:15:00</t>
+        </is>
+      </c>
+      <c r="F150" s="31" t="n">
+        <v>45715</v>
+      </c>
+      <c r="G150" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t>唐奇安破線出場</t>
+        </is>
+      </c>
+      <c r="I150" s="19" t="n">
+        <v>110</v>
+      </c>
+      <c r="J150" s="39" t="n">
+        <v>-650</v>
+      </c>
+      <c r="K150" s="40" t="n">
+        <v>-0.0007109999999999999</v>
+      </c>
+      <c r="L150" s="41" t="n">
+        <v>-14042</v>
+      </c>
+      <c r="M150" s="35" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1">
+      <c r="A151" s="5" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:05:00</t>
+        </is>
+      </c>
+      <c r="D151" s="25" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:10:00</t>
+        </is>
+      </c>
+      <c r="F151" s="25" t="n">
+        <v>45642</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H151" s="5" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I151" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="J151" s="27" t="n">
+        <v>-656</v>
+      </c>
+      <c r="K151" s="28" t="n">
+        <v>-0.001439</v>
+      </c>
+      <c r="L151" s="29" t="n">
+        <v>-14698</v>
+      </c>
+      <c r="M151" s="30" t="n">
+        <v>90452</v>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1">
+      <c r="A152" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>放空 (SELL)</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:45:00</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="n">
+        <v>45576</v>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:50:00</t>
+        </is>
+      </c>
+      <c r="F152" s="31" t="n">
+        <v>45632</v>
+      </c>
+      <c r="G152" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H152" s="8" t="inlineStr">
+        <is>
+          <t>停損 (SL)</t>
+        </is>
+      </c>
+      <c r="I152" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="J152" s="39" t="n">
+        <v>-616</v>
+      </c>
+      <c r="K152" s="40" t="n">
+        <v>-0.001352</v>
+      </c>
+      <c r="L152" s="41" t="n">
+        <v>-15314</v>
+      </c>
+      <c r="M152" s="35" t="n">
+        <v>89836</v>
       </c>
     </row>
   </sheetData>
@@ -23866,7 +25679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1752"/>
+  <dimension ref="A1:E1884"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -57160,6 +58973,2514 @@
         <v>96600</v>
       </c>
     </row>
+    <row r="1753">
+      <c r="A1753" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:10:00</t>
+        </is>
+      </c>
+      <c r="B1753" s="25" t="n">
+        <v>47090</v>
+      </c>
+      <c r="C1753" s="25" t="n">
+        <v>108155</v>
+      </c>
+      <c r="D1753" s="25" t="n">
+        <v>78563</v>
+      </c>
+      <c r="E1753" s="25" t="n">
+        <v>89430</v>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:25:00</t>
+        </is>
+      </c>
+      <c r="B1754" s="31" t="n">
+        <v>47210</v>
+      </c>
+      <c r="C1754" s="31" t="n">
+        <v>108155</v>
+      </c>
+      <c r="D1754" s="31" t="n">
+        <v>78563</v>
+      </c>
+      <c r="E1754" s="31" t="n">
+        <v>89430</v>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:40:00</t>
+        </is>
+      </c>
+      <c r="B1755" s="25" t="n">
+        <v>47304</v>
+      </c>
+      <c r="C1755" s="25" t="n">
+        <v>110015</v>
+      </c>
+      <c r="D1755" s="25" t="n">
+        <v>79493</v>
+      </c>
+      <c r="E1755" s="25" t="n">
+        <v>90360</v>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 15:55:00</t>
+        </is>
+      </c>
+      <c r="B1756" s="31" t="n">
+        <v>47316</v>
+      </c>
+      <c r="C1756" s="31" t="n">
+        <v>110255</v>
+      </c>
+      <c r="D1756" s="31" t="n">
+        <v>79613</v>
+      </c>
+      <c r="E1756" s="31" t="n">
+        <v>90480</v>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:10:00</t>
+        </is>
+      </c>
+      <c r="B1757" s="25" t="n">
+        <v>47276</v>
+      </c>
+      <c r="C1757" s="25" t="n">
+        <v>109455</v>
+      </c>
+      <c r="D1757" s="25" t="n">
+        <v>79213</v>
+      </c>
+      <c r="E1757" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:25:00</t>
+        </is>
+      </c>
+      <c r="B1758" s="31" t="n">
+        <v>47265</v>
+      </c>
+      <c r="C1758" s="31" t="n">
+        <v>109235</v>
+      </c>
+      <c r="D1758" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1758" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:40:00</t>
+        </is>
+      </c>
+      <c r="B1759" s="25" t="n">
+        <v>47192</v>
+      </c>
+      <c r="C1759" s="25" t="n">
+        <v>107775</v>
+      </c>
+      <c r="D1759" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1759" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:55:00</t>
+        </is>
+      </c>
+      <c r="B1760" s="31" t="n">
+        <v>47130</v>
+      </c>
+      <c r="C1760" s="31" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1760" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1760" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:10:00</t>
+        </is>
+      </c>
+      <c r="B1761" s="25" t="n">
+        <v>47200</v>
+      </c>
+      <c r="C1761" s="25" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1761" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1761" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:25:00</t>
+        </is>
+      </c>
+      <c r="B1762" s="31" t="n">
+        <v>47220</v>
+      </c>
+      <c r="C1762" s="31" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1762" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1762" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:40:00</t>
+        </is>
+      </c>
+      <c r="B1763" s="25" t="n">
+        <v>47241</v>
+      </c>
+      <c r="C1763" s="25" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1763" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1763" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:55:00</t>
+        </is>
+      </c>
+      <c r="B1764" s="31" t="n">
+        <v>47195</v>
+      </c>
+      <c r="C1764" s="31" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1764" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1764" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 18:10:00</t>
+        </is>
+      </c>
+      <c r="B1765" s="25" t="n">
+        <v>47121</v>
+      </c>
+      <c r="C1765" s="25" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1765" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1765" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 18:25:00</t>
+        </is>
+      </c>
+      <c r="B1766" s="31" t="n">
+        <v>47165</v>
+      </c>
+      <c r="C1766" s="31" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1766" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1766" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 18:40:00</t>
+        </is>
+      </c>
+      <c r="B1767" s="25" t="n">
+        <v>47226</v>
+      </c>
+      <c r="C1767" s="25" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1767" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1767" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 18:55:00</t>
+        </is>
+      </c>
+      <c r="B1768" s="31" t="n">
+        <v>47203</v>
+      </c>
+      <c r="C1768" s="31" t="n">
+        <v>106045</v>
+      </c>
+      <c r="D1768" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1768" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:10:00</t>
+        </is>
+      </c>
+      <c r="B1769" s="25" t="n">
+        <v>47217</v>
+      </c>
+      <c r="C1769" s="25" t="n">
+        <v>105485</v>
+      </c>
+      <c r="D1769" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1769" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:25:00</t>
+        </is>
+      </c>
+      <c r="B1770" s="31" t="n">
+        <v>47267</v>
+      </c>
+      <c r="C1770" s="31" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1770" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1770" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:40:00</t>
+        </is>
+      </c>
+      <c r="B1771" s="25" t="n">
+        <v>47281</v>
+      </c>
+      <c r="C1771" s="25" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1771" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1771" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 19:55:00</t>
+        </is>
+      </c>
+      <c r="B1772" s="31" t="n">
+        <v>47277</v>
+      </c>
+      <c r="C1772" s="31" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1772" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1772" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:10:00</t>
+        </is>
+      </c>
+      <c r="B1773" s="25" t="n">
+        <v>47268</v>
+      </c>
+      <c r="C1773" s="25" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1773" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1773" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:25:00</t>
+        </is>
+      </c>
+      <c r="B1774" s="31" t="n">
+        <v>47289</v>
+      </c>
+      <c r="C1774" s="31" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1774" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1774" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:40:00</t>
+        </is>
+      </c>
+      <c r="B1775" s="25" t="n">
+        <v>47252</v>
+      </c>
+      <c r="C1775" s="25" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1775" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1775" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:55:00</t>
+        </is>
+      </c>
+      <c r="B1776" s="31" t="n">
+        <v>47284</v>
+      </c>
+      <c r="C1776" s="31" t="n">
+        <v>106055</v>
+      </c>
+      <c r="D1776" s="31" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1776" s="31" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:10:00</t>
+        </is>
+      </c>
+      <c r="B1777" s="25" t="n">
+        <v>47344</v>
+      </c>
+      <c r="C1777" s="25" t="n">
+        <v>106135</v>
+      </c>
+      <c r="D1777" s="25" t="n">
+        <v>78937</v>
+      </c>
+      <c r="E1777" s="25" t="n">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:25:00</t>
+        </is>
+      </c>
+      <c r="B1778" s="31" t="n">
+        <v>47396</v>
+      </c>
+      <c r="C1778" s="31" t="n">
+        <v>106765</v>
+      </c>
+      <c r="D1778" s="31" t="n">
+        <v>79107</v>
+      </c>
+      <c r="E1778" s="31" t="n">
+        <v>90174</v>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:40:00</t>
+        </is>
+      </c>
+      <c r="B1779" s="25" t="n">
+        <v>47233</v>
+      </c>
+      <c r="C1779" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1779" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1779" s="25" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 21:55:00</t>
+        </is>
+      </c>
+      <c r="B1780" s="31" t="n">
+        <v>47271</v>
+      </c>
+      <c r="C1780" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1780" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1780" s="31" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 22:10:00</t>
+        </is>
+      </c>
+      <c r="B1781" s="25" t="n">
+        <v>47203</v>
+      </c>
+      <c r="C1781" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1781" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1781" s="25" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 22:25:00</t>
+        </is>
+      </c>
+      <c r="B1782" s="31" t="n">
+        <v>47270</v>
+      </c>
+      <c r="C1782" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1782" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1782" s="31" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 22:40:00</t>
+        </is>
+      </c>
+      <c r="B1783" s="25" t="n">
+        <v>47280</v>
+      </c>
+      <c r="C1783" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1783" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1783" s="25" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 22:55:00</t>
+        </is>
+      </c>
+      <c r="B1784" s="31" t="n">
+        <v>47295</v>
+      </c>
+      <c r="C1784" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1784" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1784" s="31" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 23:10:00</t>
+        </is>
+      </c>
+      <c r="B1785" s="25" t="n">
+        <v>47335</v>
+      </c>
+      <c r="C1785" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1785" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1785" s="25" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 23:25:00</t>
+        </is>
+      </c>
+      <c r="B1786" s="31" t="n">
+        <v>47356</v>
+      </c>
+      <c r="C1786" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1786" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1786" s="31" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 23:40:00</t>
+        </is>
+      </c>
+      <c r="B1787" s="25" t="n">
+        <v>47404</v>
+      </c>
+      <c r="C1787" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1787" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1787" s="25" t="n">
+        <v>89418</v>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 23:55:00</t>
+        </is>
+      </c>
+      <c r="B1788" s="31" t="n">
+        <v>47404</v>
+      </c>
+      <c r="C1788" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1788" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1788" s="31" t="n">
+        <v>89438</v>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:10:00</t>
+        </is>
+      </c>
+      <c r="B1789" s="25" t="n">
+        <v>47382</v>
+      </c>
+      <c r="C1789" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1789" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1789" s="25" t="n">
+        <v>88992</v>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:25:00</t>
+        </is>
+      </c>
+      <c r="B1790" s="31" t="n">
+        <v>47369</v>
+      </c>
+      <c r="C1790" s="31" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1790" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1790" s="31" t="n">
+        <v>88992</v>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:40:00</t>
+        </is>
+      </c>
+      <c r="B1791" s="25" t="n">
+        <v>47438</v>
+      </c>
+      <c r="C1791" s="25" t="n">
+        <v>105575</v>
+      </c>
+      <c r="D1791" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1791" s="25" t="n">
+        <v>88992</v>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 00:55:00</t>
+        </is>
+      </c>
+      <c r="B1792" s="31" t="n">
+        <v>47463</v>
+      </c>
+      <c r="C1792" s="31" t="n">
+        <v>105945</v>
+      </c>
+      <c r="D1792" s="31" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1792" s="31" t="n">
+        <v>88992</v>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:10:00</t>
+        </is>
+      </c>
+      <c r="B1793" s="25" t="n">
+        <v>47515</v>
+      </c>
+      <c r="C1793" s="25" t="n">
+        <v>105945</v>
+      </c>
+      <c r="D1793" s="25" t="n">
+        <v>78351</v>
+      </c>
+      <c r="E1793" s="25" t="n">
+        <v>88962</v>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:25:00</t>
+        </is>
+      </c>
+      <c r="B1794" s="31" t="n">
+        <v>47480</v>
+      </c>
+      <c r="C1794" s="31" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1794" s="31" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1794" s="31" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:40:00</t>
+        </is>
+      </c>
+      <c r="B1795" s="25" t="n">
+        <v>47488</v>
+      </c>
+      <c r="C1795" s="25" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1795" s="25" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1795" s="25" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 01:55:00</t>
+        </is>
+      </c>
+      <c r="B1796" s="31" t="n">
+        <v>47488</v>
+      </c>
+      <c r="C1796" s="31" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1796" s="31" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1796" s="31" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:10:00</t>
+        </is>
+      </c>
+      <c r="B1797" s="25" t="n">
+        <v>47490</v>
+      </c>
+      <c r="C1797" s="25" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1797" s="25" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1797" s="25" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:25:00</t>
+        </is>
+      </c>
+      <c r="B1798" s="31" t="n">
+        <v>47506</v>
+      </c>
+      <c r="C1798" s="31" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1798" s="31" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1798" s="31" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:40:00</t>
+        </is>
+      </c>
+      <c r="B1799" s="25" t="n">
+        <v>47537</v>
+      </c>
+      <c r="C1799" s="25" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1799" s="25" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1799" s="25" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 02:55:00</t>
+        </is>
+      </c>
+      <c r="B1800" s="31" t="n">
+        <v>47362</v>
+      </c>
+      <c r="C1800" s="31" t="n">
+        <v>105054</v>
+      </c>
+      <c r="D1800" s="31" t="n">
+        <v>77905</v>
+      </c>
+      <c r="E1800" s="31" t="n">
+        <v>88636</v>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:10:00</t>
+        </is>
+      </c>
+      <c r="B1801" s="25" t="n">
+        <v>47332</v>
+      </c>
+      <c r="C1801" s="25" t="n">
+        <v>104414</v>
+      </c>
+      <c r="D1801" s="25" t="n">
+        <v>77585</v>
+      </c>
+      <c r="E1801" s="25" t="n">
+        <v>88316</v>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:25:00</t>
+        </is>
+      </c>
+      <c r="B1802" s="31" t="n">
+        <v>47492</v>
+      </c>
+      <c r="C1802" s="31" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1802" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1802" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:40:00</t>
+        </is>
+      </c>
+      <c r="B1803" s="25" t="n">
+        <v>47479</v>
+      </c>
+      <c r="C1803" s="25" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1803" s="25" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1803" s="25" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 03:55:00</t>
+        </is>
+      </c>
+      <c r="B1804" s="31" t="n">
+        <v>47455</v>
+      </c>
+      <c r="C1804" s="31" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1804" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1804" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 04:10:00</t>
+        </is>
+      </c>
+      <c r="B1805" s="25" t="n">
+        <v>47421</v>
+      </c>
+      <c r="C1805" s="25" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1805" s="25" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1805" s="25" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 04:25:00</t>
+        </is>
+      </c>
+      <c r="B1806" s="31" t="n">
+        <v>47453</v>
+      </c>
+      <c r="C1806" s="31" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1806" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1806" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 04:40:00</t>
+        </is>
+      </c>
+      <c r="B1807" s="25" t="n">
+        <v>47487</v>
+      </c>
+      <c r="C1807" s="25" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1807" s="25" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1807" s="25" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 04:55:00</t>
+        </is>
+      </c>
+      <c r="B1808" s="31" t="n">
+        <v>47481</v>
+      </c>
+      <c r="C1808" s="31" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1808" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1808" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:50:00</t>
+        </is>
+      </c>
+      <c r="B1809" s="25" t="n">
+        <v>47277</v>
+      </c>
+      <c r="C1809" s="25" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1809" s="25" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1809" s="25" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:05:00</t>
+        </is>
+      </c>
+      <c r="B1810" s="31" t="n">
+        <v>47256</v>
+      </c>
+      <c r="C1810" s="31" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1810" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1810" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:20:00</t>
+        </is>
+      </c>
+      <c r="B1811" s="25" t="n">
+        <v>47142</v>
+      </c>
+      <c r="C1811" s="25" t="n">
+        <v>103664</v>
+      </c>
+      <c r="D1811" s="25" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1811" s="25" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:35:00</t>
+        </is>
+      </c>
+      <c r="B1812" s="31" t="n">
+        <v>47020</v>
+      </c>
+      <c r="C1812" s="31" t="n">
+        <v>106004</v>
+      </c>
+      <c r="D1812" s="31" t="n">
+        <v>77209</v>
+      </c>
+      <c r="E1812" s="31" t="n">
+        <v>87940</v>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:50:00</t>
+        </is>
+      </c>
+      <c r="B1813" s="25" t="n">
+        <v>46950</v>
+      </c>
+      <c r="C1813" s="25" t="n">
+        <v>107404</v>
+      </c>
+      <c r="D1813" s="25" t="n">
+        <v>78119</v>
+      </c>
+      <c r="E1813" s="25" t="n">
+        <v>88850</v>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:05:00</t>
+        </is>
+      </c>
+      <c r="B1814" s="31" t="n">
+        <v>46925</v>
+      </c>
+      <c r="C1814" s="31" t="n">
+        <v>107904</v>
+      </c>
+      <c r="D1814" s="31" t="n">
+        <v>78369</v>
+      </c>
+      <c r="E1814" s="31" t="n">
+        <v>89100</v>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:20:00</t>
+        </is>
+      </c>
+      <c r="B1815" s="25" t="n">
+        <v>46944</v>
+      </c>
+      <c r="C1815" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1815" s="25" t="n">
+        <v>78179</v>
+      </c>
+      <c r="E1815" s="25" t="n">
+        <v>88910</v>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:35:00</t>
+        </is>
+      </c>
+      <c r="B1816" s="31" t="n">
+        <v>46923</v>
+      </c>
+      <c r="C1816" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1816" s="31" t="n">
+        <v>78389</v>
+      </c>
+      <c r="E1816" s="31" t="n">
+        <v>89120</v>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:50:00</t>
+        </is>
+      </c>
+      <c r="B1817" s="25" t="n">
+        <v>46811</v>
+      </c>
+      <c r="C1817" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1817" s="25" t="n">
+        <v>79509</v>
+      </c>
+      <c r="E1817" s="25" t="n">
+        <v>90240</v>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:05:00</t>
+        </is>
+      </c>
+      <c r="B1818" s="31" t="n">
+        <v>46843</v>
+      </c>
+      <c r="C1818" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1818" s="31" t="n">
+        <v>79189</v>
+      </c>
+      <c r="E1818" s="31" t="n">
+        <v>89920</v>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:20:00</t>
+        </is>
+      </c>
+      <c r="B1819" s="25" t="n">
+        <v>46802</v>
+      </c>
+      <c r="C1819" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1819" s="25" t="n">
+        <v>79599</v>
+      </c>
+      <c r="E1819" s="25" t="n">
+        <v>90330</v>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:35:00</t>
+        </is>
+      </c>
+      <c r="B1820" s="31" t="n">
+        <v>46676</v>
+      </c>
+      <c r="C1820" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1820" s="31" t="n">
+        <v>80859</v>
+      </c>
+      <c r="E1820" s="31" t="n">
+        <v>91590</v>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:50:00</t>
+        </is>
+      </c>
+      <c r="B1821" s="25" t="n">
+        <v>46534</v>
+      </c>
+      <c r="C1821" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1821" s="25" t="n">
+        <v>82279</v>
+      </c>
+      <c r="E1821" s="25" t="n">
+        <v>93010</v>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:05:00</t>
+        </is>
+      </c>
+      <c r="B1822" s="31" t="n">
+        <v>46540</v>
+      </c>
+      <c r="C1822" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1822" s="31" t="n">
+        <v>82219</v>
+      </c>
+      <c r="E1822" s="31" t="n">
+        <v>92950</v>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:20:00</t>
+        </is>
+      </c>
+      <c r="B1823" s="25" t="n">
+        <v>46518</v>
+      </c>
+      <c r="C1823" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1823" s="25" t="n">
+        <v>82439</v>
+      </c>
+      <c r="E1823" s="25" t="n">
+        <v>93170</v>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:35:00</t>
+        </is>
+      </c>
+      <c r="B1824" s="31" t="n">
+        <v>46463</v>
+      </c>
+      <c r="C1824" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1824" s="31" t="n">
+        <v>82989</v>
+      </c>
+      <c r="E1824" s="31" t="n">
+        <v>93720</v>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:50:00</t>
+        </is>
+      </c>
+      <c r="B1825" s="25" t="n">
+        <v>46408</v>
+      </c>
+      <c r="C1825" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1825" s="25" t="n">
+        <v>83539</v>
+      </c>
+      <c r="E1825" s="25" t="n">
+        <v>94270</v>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 13:05:00</t>
+        </is>
+      </c>
+      <c r="B1826" s="31" t="n">
+        <v>46440</v>
+      </c>
+      <c r="C1826" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1826" s="31" t="n">
+        <v>83219</v>
+      </c>
+      <c r="E1826" s="31" t="n">
+        <v>93950</v>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 13:20:00</t>
+        </is>
+      </c>
+      <c r="B1827" s="25" t="n">
+        <v>46340</v>
+      </c>
+      <c r="C1827" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1827" s="25" t="n">
+        <v>84219</v>
+      </c>
+      <c r="E1827" s="25" t="n">
+        <v>94950</v>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 13:35:00</t>
+        </is>
+      </c>
+      <c r="B1828" s="31" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C1828" s="31" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1828" s="31" t="n">
+        <v>84719</v>
+      </c>
+      <c r="E1828" s="31" t="n">
+        <v>95450</v>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:05:00</t>
+        </is>
+      </c>
+      <c r="B1829" s="25" t="n">
+        <v>46208</v>
+      </c>
+      <c r="C1829" s="25" t="n">
+        <v>108054</v>
+      </c>
+      <c r="D1829" s="25" t="n">
+        <v>85539</v>
+      </c>
+      <c r="E1829" s="25" t="n">
+        <v>96270</v>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:20:00</t>
+        </is>
+      </c>
+      <c r="B1830" s="31" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C1830" s="31" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1830" s="31" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1830" s="31" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:35:00</t>
+        </is>
+      </c>
+      <c r="B1831" s="25" t="n">
+        <v>46298</v>
+      </c>
+      <c r="C1831" s="25" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1831" s="25" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1831" s="25" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 15:50:00</t>
+        </is>
+      </c>
+      <c r="B1832" s="31" t="n">
+        <v>46271</v>
+      </c>
+      <c r="C1832" s="31" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1832" s="31" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1832" s="31" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:05:00</t>
+        </is>
+      </c>
+      <c r="B1833" s="25" t="n">
+        <v>46214</v>
+      </c>
+      <c r="C1833" s="25" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1833" s="25" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1833" s="25" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:20:00</t>
+        </is>
+      </c>
+      <c r="B1834" s="31" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C1834" s="31" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1834" s="31" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1834" s="31" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:35:00</t>
+        </is>
+      </c>
+      <c r="B1835" s="25" t="n">
+        <v>46213</v>
+      </c>
+      <c r="C1835" s="25" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1835" s="25" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1835" s="25" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:50:00</t>
+        </is>
+      </c>
+      <c r="B1836" s="31" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C1836" s="31" t="n">
+        <v>107024</v>
+      </c>
+      <c r="D1836" s="31" t="n">
+        <v>84573</v>
+      </c>
+      <c r="E1836" s="31" t="n">
+        <v>95304</v>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:05:00</t>
+        </is>
+      </c>
+      <c r="B1837" s="25" t="n">
+        <v>46085</v>
+      </c>
+      <c r="C1837" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1837" s="25" t="n">
+        <v>84223</v>
+      </c>
+      <c r="E1837" s="25" t="n">
+        <v>94604</v>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:20:00</t>
+        </is>
+      </c>
+      <c r="B1838" s="31" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C1838" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1838" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1838" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:35:00</t>
+        </is>
+      </c>
+      <c r="B1839" s="25" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C1839" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1839" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1839" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:50:00</t>
+        </is>
+      </c>
+      <c r="B1840" s="31" t="n">
+        <v>46134</v>
+      </c>
+      <c r="C1840" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1840" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1840" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:05:00</t>
+        </is>
+      </c>
+      <c r="B1841" s="25" t="n">
+        <v>46207</v>
+      </c>
+      <c r="C1841" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1841" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1841" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:20:00</t>
+        </is>
+      </c>
+      <c r="B1842" s="31" t="n">
+        <v>46233</v>
+      </c>
+      <c r="C1842" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1842" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1842" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:35:00</t>
+        </is>
+      </c>
+      <c r="B1843" s="25" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C1843" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1843" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1843" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:50:00</t>
+        </is>
+      </c>
+      <c r="B1844" s="31" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C1844" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1844" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1844" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:05:00</t>
+        </is>
+      </c>
+      <c r="B1845" s="25" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C1845" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1845" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1845" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:20:00</t>
+        </is>
+      </c>
+      <c r="B1846" s="31" t="n">
+        <v>46150</v>
+      </c>
+      <c r="C1846" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1846" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1846" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:35:00</t>
+        </is>
+      </c>
+      <c r="B1847" s="25" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C1847" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1847" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1847" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 19:50:00</t>
+        </is>
+      </c>
+      <c r="B1848" s="31" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C1848" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1848" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1848" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:05:00</t>
+        </is>
+      </c>
+      <c r="B1849" s="25" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C1849" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1849" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1849" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:20:00</t>
+        </is>
+      </c>
+      <c r="B1850" s="31" t="n">
+        <v>46250</v>
+      </c>
+      <c r="C1850" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1850" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1850" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:35:00</t>
+        </is>
+      </c>
+      <c r="B1851" s="25" t="n">
+        <v>46200</v>
+      </c>
+      <c r="C1851" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1851" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1851" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:50:00</t>
+        </is>
+      </c>
+      <c r="B1852" s="31" t="n">
+        <v>46187</v>
+      </c>
+      <c r="C1852" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1852" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1852" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:05:00</t>
+        </is>
+      </c>
+      <c r="B1853" s="25" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C1853" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1853" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1853" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:20:00</t>
+        </is>
+      </c>
+      <c r="B1854" s="31" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C1854" s="31" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1854" s="31" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1854" s="31" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:35:00</t>
+        </is>
+      </c>
+      <c r="B1855" s="25" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C1855" s="25" t="n">
+        <v>106214</v>
+      </c>
+      <c r="D1855" s="25" t="n">
+        <v>82747</v>
+      </c>
+      <c r="E1855" s="25" t="n">
+        <v>91654</v>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:50:00</t>
+        </is>
+      </c>
+      <c r="B1856" s="31" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C1856" s="31" t="n">
+        <v>104524</v>
+      </c>
+      <c r="D1856" s="31" t="n">
+        <v>81901</v>
+      </c>
+      <c r="E1856" s="31" t="n">
+        <v>89964</v>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:05:00</t>
+        </is>
+      </c>
+      <c r="B1857" s="25" t="n">
+        <v>46232</v>
+      </c>
+      <c r="C1857" s="25" t="n">
+        <v>104524</v>
+      </c>
+      <c r="D1857" s="25" t="n">
+        <v>81901</v>
+      </c>
+      <c r="E1857" s="25" t="n">
+        <v>89964</v>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:20:00</t>
+        </is>
+      </c>
+      <c r="B1858" s="31" t="n">
+        <v>46085</v>
+      </c>
+      <c r="C1858" s="31" t="n">
+        <v>104524</v>
+      </c>
+      <c r="D1858" s="31" t="n">
+        <v>81901</v>
+      </c>
+      <c r="E1858" s="31" t="n">
+        <v>89964</v>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:35:00</t>
+        </is>
+      </c>
+      <c r="B1859" s="25" t="n">
+        <v>45958</v>
+      </c>
+      <c r="C1859" s="25" t="n">
+        <v>106904</v>
+      </c>
+      <c r="D1859" s="25" t="n">
+        <v>83091</v>
+      </c>
+      <c r="E1859" s="25" t="n">
+        <v>91154</v>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 22:50:00</t>
+        </is>
+      </c>
+      <c r="B1860" s="31" t="n">
+        <v>45860</v>
+      </c>
+      <c r="C1860" s="31" t="n">
+        <v>108864</v>
+      </c>
+      <c r="D1860" s="31" t="n">
+        <v>84071</v>
+      </c>
+      <c r="E1860" s="31" t="n">
+        <v>92134</v>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:05:00</t>
+        </is>
+      </c>
+      <c r="B1861" s="25" t="n">
+        <v>45795</v>
+      </c>
+      <c r="C1861" s="25" t="n">
+        <v>110164</v>
+      </c>
+      <c r="D1861" s="25" t="n">
+        <v>84721</v>
+      </c>
+      <c r="E1861" s="25" t="n">
+        <v>92784</v>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:20:00</t>
+        </is>
+      </c>
+      <c r="B1862" s="31" t="n">
+        <v>45892</v>
+      </c>
+      <c r="C1862" s="31" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1862" s="31" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1862" s="31" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:35:00</t>
+        </is>
+      </c>
+      <c r="B1863" s="25" t="n">
+        <v>45803</v>
+      </c>
+      <c r="C1863" s="25" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1863" s="25" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1863" s="25" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 23:50:00</t>
+        </is>
+      </c>
+      <c r="B1864" s="31" t="n">
+        <v>45844</v>
+      </c>
+      <c r="C1864" s="31" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1864" s="31" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1864" s="31" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:05:00</t>
+        </is>
+      </c>
+      <c r="B1865" s="25" t="n">
+        <v>45943</v>
+      </c>
+      <c r="C1865" s="25" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1865" s="25" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1865" s="25" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:20:00</t>
+        </is>
+      </c>
+      <c r="B1866" s="31" t="n">
+        <v>45918</v>
+      </c>
+      <c r="C1866" s="31" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1866" s="31" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1866" s="31" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:35:00</t>
+        </is>
+      </c>
+      <c r="B1867" s="25" t="n">
+        <v>45808</v>
+      </c>
+      <c r="C1867" s="25" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1867" s="25" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1867" s="25" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 00:50:00</t>
+        </is>
+      </c>
+      <c r="B1868" s="31" t="n">
+        <v>45691</v>
+      </c>
+      <c r="C1868" s="31" t="n">
+        <v>110834</v>
+      </c>
+      <c r="D1868" s="31" t="n">
+        <v>83695</v>
+      </c>
+      <c r="E1868" s="31" t="n">
+        <v>91758</v>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:05:00</t>
+        </is>
+      </c>
+      <c r="B1869" s="25" t="n">
+        <v>45657</v>
+      </c>
+      <c r="C1869" s="25" t="n">
+        <v>110204</v>
+      </c>
+      <c r="D1869" s="25" t="n">
+        <v>84005</v>
+      </c>
+      <c r="E1869" s="25" t="n">
+        <v>92378</v>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:20:00</t>
+        </is>
+      </c>
+      <c r="B1870" s="31" t="n">
+        <v>45715</v>
+      </c>
+      <c r="C1870" s="31" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1870" s="31" t="n">
+        <v>83425</v>
+      </c>
+      <c r="E1870" s="31" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:35:00</t>
+        </is>
+      </c>
+      <c r="B1871" s="25" t="n">
+        <v>45743</v>
+      </c>
+      <c r="C1871" s="25" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1871" s="25" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1871" s="25" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 01:50:00</t>
+        </is>
+      </c>
+      <c r="B1872" s="31" t="n">
+        <v>45706</v>
+      </c>
+      <c r="C1872" s="31" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1872" s="31" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1872" s="31" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 02:05:00</t>
+        </is>
+      </c>
+      <c r="B1873" s="25" t="n">
+        <v>45665</v>
+      </c>
+      <c r="C1873" s="25" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1873" s="25" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1873" s="25" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 02:20:00</t>
+        </is>
+      </c>
+      <c r="B1874" s="31" t="n">
+        <v>45739</v>
+      </c>
+      <c r="C1874" s="31" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1874" s="31" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1874" s="31" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 02:35:00</t>
+        </is>
+      </c>
+      <c r="B1875" s="25" t="n">
+        <v>45660</v>
+      </c>
+      <c r="C1875" s="25" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1875" s="25" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1875" s="25" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 02:50:00</t>
+        </is>
+      </c>
+      <c r="B1876" s="31" t="n">
+        <v>45629</v>
+      </c>
+      <c r="C1876" s="31" t="n">
+        <v>108754</v>
+      </c>
+      <c r="D1876" s="31" t="n">
+        <v>82809</v>
+      </c>
+      <c r="E1876" s="31" t="n">
+        <v>91108</v>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:05:00</t>
+        </is>
+      </c>
+      <c r="B1877" s="25" t="n">
+        <v>45585</v>
+      </c>
+      <c r="C1877" s="25" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1877" s="25" t="n">
+        <v>82779</v>
+      </c>
+      <c r="E1877" s="25" t="n">
+        <v>91078</v>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:20:00</t>
+        </is>
+      </c>
+      <c r="B1878" s="31" t="n">
+        <v>45677</v>
+      </c>
+      <c r="C1878" s="31" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1878" s="31" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1878" s="31" t="n">
+        <v>90452</v>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:35:00</t>
+        </is>
+      </c>
+      <c r="B1879" s="25" t="n">
+        <v>45579</v>
+      </c>
+      <c r="C1879" s="25" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1879" s="25" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1879" s="25" t="n">
+        <v>90452</v>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:50:00</t>
+        </is>
+      </c>
+      <c r="B1880" s="31" t="n">
+        <v>45693</v>
+      </c>
+      <c r="C1880" s="31" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1880" s="31" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1880" s="31" t="n">
+        <v>89836</v>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:05:00</t>
+        </is>
+      </c>
+      <c r="B1881" s="25" t="n">
+        <v>45666</v>
+      </c>
+      <c r="C1881" s="25" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1881" s="25" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1881" s="25" t="n">
+        <v>89836</v>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:20:00</t>
+        </is>
+      </c>
+      <c r="B1882" s="31" t="n">
+        <v>45655</v>
+      </c>
+      <c r="C1882" s="31" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1882" s="31" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1882" s="31" t="n">
+        <v>89836</v>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:35:00</t>
+        </is>
+      </c>
+      <c r="B1883" s="25" t="n">
+        <v>45637</v>
+      </c>
+      <c r="C1883" s="25" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1883" s="25" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1883" s="25" t="n">
+        <v>89836</v>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:50:00</t>
+        </is>
+      </c>
+      <c r="B1884" s="31" t="n">
+        <v>45638</v>
+      </c>
+      <c r="C1884" s="31" t="n">
+        <v>108584</v>
+      </c>
+      <c r="D1884" s="31" t="n">
+        <v>82153</v>
+      </c>
+      <c r="E1884" s="31" t="n">
+        <v>89836</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>